<commit_message>
Update latest provided by IA
</commit_message>
<xml_diff>
--- a/input/requirements/Procedure.xlsx
+++ b/input/requirements/Procedure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TessavanAlphen\Projects\GBB-IG\input\requirements\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahenket/Development/GitHub/Nictiz/GBB-IG/input/requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E763DAFF-1EFF-401A-84AC-F527979C6F1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{20572DD5-0653-6B41-AC4F-00D5B12D1465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34560" windowHeight="21660" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -216,7 +216,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="562" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="403">
   <si>
     <t>Veld</t>
   </si>
@@ -1441,6 +1441,12 @@
   <si>
     <t>1..1
 Verplicht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De reden waarom de procedure is uitgevoerd of de indicatie van de verrichtign. </t>
+  </si>
+  <si>
+    <t>Dit kan een begrip uit een terminologie zijn of een verwijzing naar een specifieke instantie die de reden/indicatie beschrijft.</t>
   </si>
 </sst>
 </file>
@@ -2697,12 +2703,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F1013F7-63B2-4F83-92B0-1C8153859891}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="218.44140625" customWidth="1"/>
+    <col min="1" max="1" width="218.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
     </row>
   </sheetData>
@@ -2714,18 +2720,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC1E3B3-D087-4A2B-920B-9BA971FAD64B}">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="190.95" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="191" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
     <col min="2" max="2" width="59.6640625" customWidth="1"/>
-    <col min="3" max="3" width="58.44140625" style="3" customWidth="1"/>
-    <col min="4" max="4" width="99.77734375" style="3" customWidth="1"/>
+    <col min="3" max="3" width="58.5" style="3" customWidth="1"/>
+    <col min="4" max="4" width="99.83203125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="190.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="191" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3"/>
     </row>
-    <row r="2" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="15" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -2733,7 +2739,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2741,7 +2747,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="96" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -2749,7 +2755,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -2757,7 +2763,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2765,7 +2771,7 @@
         <v>337</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="48" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2773,7 +2779,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="32" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -2781,7 +2787,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="80" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -2792,7 +2798,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="72" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="64" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -2803,7 +2809,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>335</v>
       </c>
@@ -2821,20 +2827,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
   <dimension ref="A1:K77"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="22.44140625" style="4" customWidth="1"/>
-    <col min="3" max="3" width="14.77734375" style="4" customWidth="1"/>
+    <col min="1" max="2" width="22.5" style="4" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" style="4" customWidth="1"/>
     <col min="4" max="4" width="17" style="4" customWidth="1"/>
     <col min="5" max="5" width="38" customWidth="1"/>
-    <col min="6" max="6" width="68.44140625" customWidth="1"/>
-    <col min="7" max="7" width="52.109375" customWidth="1"/>
+    <col min="6" max="6" width="68.5" customWidth="1"/>
+    <col min="7" max="7" width="52.1640625" customWidth="1"/>
     <col min="8" max="9" width="48.6640625" customWidth="1"/>
-    <col min="10" max="10" width="34.44140625" customWidth="1"/>
+    <col min="10" max="10" width="34.5" customWidth="1"/>
     <col min="11" max="11" width="19.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="88.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="88.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="11"/>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -2843,7 +2849,7 @@
       <c r="F1" s="11"/>
       <c r="G1" s="11"/>
     </row>
-    <row r="2" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>16</v>
       </c>
@@ -2876,7 +2882,7 @@
       </c>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A3" s="11">
         <v>0</v>
       </c>
@@ -2901,7 +2907,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A4" s="13">
         <v>1</v>
       </c>
@@ -2924,7 +2930,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A5" s="13" t="s">
         <v>30</v>
       </c>
@@ -2951,7 +2957,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A6" s="13" t="s">
         <v>34</v>
       </c>
@@ -2978,7 +2984,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A7" s="13" t="s">
         <v>38</v>
       </c>
@@ -3005,7 +3011,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="64" x14ac:dyDescent="0.2">
       <c r="A8" s="13" t="s">
         <v>43</v>
       </c>
@@ -3030,7 +3036,7 @@
       </c>
       <c r="J8" s="3"/>
     </row>
-    <row r="9" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="48" x14ac:dyDescent="0.2">
       <c r="A9" s="13" t="s">
         <v>48</v>
       </c>
@@ -3057,7 +3063,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="13" t="s">
         <v>53</v>
       </c>
@@ -3084,7 +3090,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="13" t="s">
         <v>58</v>
       </c>
@@ -3108,7 +3114,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="11" t="s">
         <v>63</v>
       </c>
@@ -3140,7 +3146,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A13" s="13" t="s">
         <v>341</v>
       </c>
@@ -3167,7 +3173,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A14" s="11">
         <v>2</v>
       </c>
@@ -3190,7 +3196,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A15" s="11" t="s">
         <v>77</v>
       </c>
@@ -3213,7 +3219,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A16" s="11" t="s">
         <v>80</v>
       </c>
@@ -3236,7 +3242,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
         <v>83</v>
       </c>
@@ -3259,7 +3265,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="11">
         <v>3</v>
       </c>
@@ -3279,7 +3285,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A19" s="11" t="s">
         <v>88</v>
       </c>
@@ -3306,7 +3312,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A20" s="11" t="s">
         <v>94</v>
       </c>
@@ -3331,7 +3337,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A21" s="11" t="s">
         <v>99</v>
       </c>
@@ -3358,7 +3364,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A22" s="11" t="s">
         <v>104</v>
       </c>
@@ -3383,7 +3389,7 @@
       </c>
       <c r="J22" s="3"/>
     </row>
-    <row r="23" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A23" s="13">
         <v>4</v>
       </c>
@@ -3406,7 +3412,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A24" s="13" t="s">
         <v>112</v>
       </c>
@@ -3433,7 +3439,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A25" s="13" t="s">
         <v>118</v>
       </c>
@@ -3456,7 +3462,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="13" t="s">
         <v>121</v>
       </c>
@@ -3479,7 +3485,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A27" s="13" t="s">
         <v>124</v>
       </c>
@@ -3502,7 +3508,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A28" s="13" t="s">
         <v>128</v>
       </c>
@@ -3525,7 +3531,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A29" s="13" t="s">
         <v>132</v>
       </c>
@@ -3548,7 +3554,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A30" s="13" t="s">
         <v>136</v>
       </c>
@@ -3571,7 +3577,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A31" s="13" t="s">
         <v>139</v>
       </c>
@@ -3594,7 +3600,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A32" s="13" t="s">
         <v>144</v>
       </c>
@@ -3617,7 +3623,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A33" s="13" t="s">
         <v>148</v>
       </c>
@@ -3640,7 +3646,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A34" s="13" t="s">
         <v>152</v>
       </c>
@@ -3663,7 +3669,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A35" s="13" t="s">
         <v>156</v>
       </c>
@@ -3686,7 +3692,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A36" s="13" t="s">
         <v>160</v>
       </c>
@@ -3709,7 +3715,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A37" s="13" t="s">
         <v>164</v>
       </c>
@@ -3732,7 +3738,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A38" s="13" t="s">
         <v>168</v>
       </c>
@@ -3755,7 +3761,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A39" s="13" t="s">
         <v>172</v>
       </c>
@@ -3778,7 +3784,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A40" s="13" t="s">
         <v>176</v>
       </c>
@@ -3801,7 +3807,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A41" s="13" t="s">
         <v>180</v>
       </c>
@@ -3824,7 +3830,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A42" s="13" t="s">
         <v>184</v>
       </c>
@@ -3847,7 +3853,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="13" t="s">
         <v>188</v>
       </c>
@@ -3870,7 +3876,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="13" t="s">
         <v>192</v>
       </c>
@@ -3897,7 +3903,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A45" s="13"/>
       <c r="B45" s="13" t="s">
         <v>64</v>
@@ -3927,7 +3933,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="46" spans="1:10" s="5" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" s="5" customFormat="1" ht="32" x14ac:dyDescent="0.2">
       <c r="A46" s="11"/>
       <c r="B46" s="13" t="s">
         <v>64</v>
@@ -3957,7 +3963,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="47" spans="1:10" s="5" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" s="5" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A47" s="13">
         <v>5</v>
       </c>
@@ -3984,7 +3990,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A48" s="14" t="s">
         <v>205</v>
       </c>
@@ -4010,7 +4016,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A49" s="14" t="s">
         <v>209</v>
       </c>
@@ -4032,7 +4038,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A50" s="13">
         <v>6</v>
       </c>
@@ -4059,7 +4065,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A51" s="11">
         <v>7</v>
       </c>
@@ -4069,12 +4075,20 @@
       <c r="E51" s="11" t="s">
         <v>219</v>
       </c>
-      <c r="G51" s="11"/>
+      <c r="F51" t="s">
+        <v>401</v>
+      </c>
+      <c r="G51" s="11" t="s">
+        <v>402</v>
+      </c>
+      <c r="H51" s="3" t="s">
+        <v>390</v>
+      </c>
       <c r="J51" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A52" s="11" t="s">
         <v>220</v>
       </c>
@@ -4101,7 +4115,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A53" s="15" t="s">
         <v>225</v>
       </c>
@@ -4128,7 +4142,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="54" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A54" s="11">
         <v>8</v>
       </c>
@@ -4155,7 +4169,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="13">
         <v>9</v>
       </c>
@@ -4182,7 +4196,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="11" t="s">
         <v>239</v>
       </c>
@@ -4212,7 +4226,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A57" s="11" t="s">
         <v>244</v>
       </c>
@@ -4244,7 +4258,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="11" t="s">
         <v>248</v>
       </c>
@@ -4274,7 +4288,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="11">
         <v>10</v>
       </c>
@@ -4301,7 +4315,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="13" t="s">
         <v>257</v>
       </c>
@@ -4329,7 +4343,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A61" s="11" t="s">
         <v>261</v>
       </c>
@@ -4357,7 +4371,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="62" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A62" s="11" t="s">
         <v>264</v>
       </c>
@@ -4385,7 +4399,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="63" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" s="11">
         <v>11</v>
       </c>
@@ -4412,7 +4426,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="64" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A64" s="11">
         <v>13</v>
       </c>
@@ -4439,7 +4453,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="65" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" ht="64" x14ac:dyDescent="0.2">
       <c r="A65" s="11">
         <v>14</v>
       </c>
@@ -4466,7 +4480,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="66" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A66" s="11">
         <v>15</v>
       </c>
@@ -4493,7 +4507,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="67" spans="1:10" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A67" s="11">
         <v>16</v>
       </c>
@@ -4520,7 +4534,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="68" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A68" s="11">
         <v>17</v>
       </c>
@@ -4547,7 +4561,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="69" spans="1:10" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" ht="48" x14ac:dyDescent="0.2">
       <c r="A69" s="11">
         <v>18</v>
       </c>
@@ -4574,7 +4588,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="70" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" ht="37.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="11">
         <v>19</v>
       </c>
@@ -4599,7 +4613,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="71" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="11" t="s">
         <v>308</v>
       </c>
@@ -4626,7 +4640,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="13">
         <v>20</v>
       </c>
@@ -4647,7 +4661,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="73" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="11">
         <v>21</v>
       </c>
@@ -4668,7 +4682,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="74" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="11">
         <v>22</v>
       </c>
@@ -4690,7 +4704,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="75" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="11"/>
       <c r="B75" s="13"/>
       <c r="C75" s="13"/>
@@ -4698,13 +4712,13 @@
       <c r="F75" s="11"/>
       <c r="G75" s="13"/>
     </row>
-    <row r="76" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F76" s="11"/>
       <c r="G76" s="13" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="77" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D77" s="13"/>
       <c r="F77" s="11"/>
       <c r="G77" s="11"/>
@@ -4720,18 +4734,18 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{273AFAA3-99F7-4E93-9580-DCAE2B14D938}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.33203125" customWidth="1"/>
-    <col min="2" max="2" width="18.44140625" customWidth="1"/>
-    <col min="3" max="3" width="14.77734375" customWidth="1"/>
-    <col min="4" max="4" width="15.109375" customWidth="1"/>
+    <col min="2" max="2" width="18.5" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.1640625" customWidth="1"/>
     <col min="5" max="5" width="16.6640625" customWidth="1"/>
-    <col min="6" max="6" width="16.44140625" customWidth="1"/>
-    <col min="7" max="7" width="41.44140625" customWidth="1"/>
+    <col min="6" max="6" width="16.5" customWidth="1"/>
+    <col min="7" max="7" width="41.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="195.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>313</v>
       </c>
@@ -4754,7 +4768,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>315</v>
       </c>
@@ -4777,7 +4791,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" ht="64" x14ac:dyDescent="0.2">
       <c r="C3" t="s">
         <v>274</v>
       </c>
@@ -4794,7 +4808,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="C4" t="s">
         <v>323</v>
       </c>
@@ -4811,7 +4825,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="C5" t="s">
         <v>326</v>
       </c>
@@ -4828,7 +4842,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="48" x14ac:dyDescent="0.2">
       <c r="C6" s="7" t="s">
         <v>328</v>
       </c>
@@ -4845,7 +4859,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.2">
       <c r="C7" t="s">
         <v>329</v>
       </c>
@@ -4872,20 +4886,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2489EBC-5098-4697-9724-F190D24E1C3D}">
   <dimension ref="A1:A5"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="111" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="111" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>332</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>334</v>
       </c>
@@ -4897,6 +4911,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -5103,7 +5128,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -5112,18 +5137,24 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{226BE694-A00C-4E31-A532-690E39C51D9D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5142,21 +5173,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6E3A9028-3436-4B29-A420-9ED5B8A085B1}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
-    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>